<commit_message>
Testing fitting xi with rho PR, exponential gives best results if xi is y and rho PR is x but, still provides error at high density (low xH2). Hence better to interpolate, though more intensive
</commit_message>
<xml_diff>
--- a/results/cal_250725_PR/calResults.xlsx
+++ b/results/cal_250725_PR/calResults.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -10,17 +10,17 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="1" documentId="11_1357E617CF19DF7F2B1B3B26FE012D16D10A0B41" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{018C2BF4-DA90-4078-BF9D-CC816F2F7758}"/>
   <bookViews>
-    <workbookView xWindow="1200" yWindow="1695" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1200" yWindow="1695" windowWidth="21600" windowHeight="11295"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="110" uniqueCount="24">
   <si>
     <t>Fluid</t>
   </si>
@@ -97,8 +97,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -112,7 +112,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -120,12 +120,14 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -144,7 +146,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -295,7 +297,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -319,9 +321,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -345,7 +347,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -380,7 +382,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -398,7 +400,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -423,7 +425,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -459,1144 +461,1149 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.5703125" customWidth="1"/>
-    <col min="2" max="2" width="6.140625" customWidth="1"/>
-    <col min="3" max="4" width="6.85546875" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" customWidth="1"/>
-    <col min="6" max="6" width="8.7109375" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
-    <col min="8" max="8" width="13.7109375" customWidth="1"/>
-    <col min="9" max="11" width="11.7109375" customWidth="1"/>
-    <col min="12" max="13" width="15" customWidth="1"/>
-    <col min="14" max="14" width="12.7109375" customWidth="1"/>
-    <col min="15" max="15" width="11.7109375" customWidth="1"/>
-    <col min="16" max="17" width="12.7109375" customWidth="1"/>
-    <col min="18" max="18" width="13.7109375" customWidth="1"/>
-    <col min="19" max="19" width="12.7109375" customWidth="1"/>
+    <col min="1" max="1" width="5.5703125" customWidth="true"/>
+    <col min="2" max="2" width="6.140625" customWidth="true"/>
+    <col min="3" max="3" width="6.85546875" customWidth="true"/>
+    <col min="5" max="5" width="10.7109375" customWidth="true"/>
+    <col min="6" max="6" width="8.7109375" customWidth="true"/>
+    <col min="7" max="7" width="12" customWidth="true"/>
+    <col min="8" max="8" width="13.7109375" customWidth="true"/>
+    <col min="9" max="9" width="11.7109375" customWidth="true"/>
+    <col min="12" max="12" width="15" customWidth="true"/>
+    <col min="14" max="14" width="12.7109375" customWidth="true"/>
+    <col min="15" max="15" width="11.7109375" customWidth="true"/>
+    <col min="16" max="16" width="12.7109375" customWidth="true"/>
+    <col min="18" max="18" width="13.7109375" customWidth="true"/>
+    <col min="19" max="19" width="12.7109375" customWidth="true"/>
+    <col min="4" max="4" width="6.85546875" customWidth="true"/>
+    <col min="10" max="10" width="11.7109375" customWidth="true"/>
+    <col min="11" max="11" width="11.7109375" customWidth="true"/>
+    <col min="13" max="13" width="15" customWidth="true"/>
+    <col min="17" max="17" width="12.7109375" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="0" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.25">
+      <c r="A2" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>32</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>14.7</v>
-      </c>
-      <c r="E2">
+      <c r="B2" s="0">
+        <v>32</v>
+      </c>
+      <c r="C2" s="0">
+        <v>0</v>
+      </c>
+      <c r="D2" s="0">
+        <v>14.699999999999999</v>
+      </c>
+      <c r="E2" s="0">
         <v>1.0135649999999998</v>
       </c>
-      <c r="F2">
-        <v>7.9399999999999998E-2</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="F2" s="0">
+        <v>0.079399999999999998</v>
+      </c>
+      <c r="G2" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="0">
         <v>14.814216867469868</v>
       </c>
-      <c r="I2">
+      <c r="I2" s="0">
         <v>5.9043386746987991</v>
       </c>
-      <c r="J2">
+      <c r="J2" s="0">
         <v>5.194539771184326</v>
       </c>
-      <c r="K2">
+      <c r="K2" s="0">
         <v>32.636798899910957</v>
       </c>
-      <c r="L2">
+      <c r="L2" s="0">
         <v>37.275903614457775</v>
       </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2">
+      <c r="M2" s="0">
+        <v>0</v>
+      </c>
+      <c r="N2" s="0">
         <v>23.22926984154881</v>
       </c>
-      <c r="O2">
+      <c r="O2" s="0">
         <v>3.7086947526174674</v>
       </c>
-      <c r="P2">
+      <c r="P2" s="0">
         <v>1.5880534763159093</v>
       </c>
-      <c r="Q2">
+      <c r="Q2" s="0">
         <v>0.43723303558108212</v>
       </c>
-      <c r="R2">
+      <c r="R2" s="0">
         <v>42.501421221852155</v>
       </c>
-      <c r="S2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="S2" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.25">
+      <c r="A3" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="B3">
-        <v>32</v>
-      </c>
-      <c r="C3">
+      <c r="B3" s="0">
+        <v>32</v>
+      </c>
+      <c r="C3" s="0">
         <v>50</v>
       </c>
-      <c r="D3">
-        <v>64.7</v>
-      </c>
-      <c r="E3">
+      <c r="D3" s="0">
+        <v>64.700000000000003</v>
+      </c>
+      <c r="E3" s="0">
         <v>4.4610649999999996</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="0">
         <v>0.3175</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="0">
         <v>48.74437869822485</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="0">
         <v>5.1064763313609474</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="0">
         <v>5.8952419652353418</v>
       </c>
-      <c r="K3">
+      <c r="K3" s="0">
         <v>32.544644448389754</v>
       </c>
-      <c r="L3">
+      <c r="L3" s="0">
         <v>85.706213017751594</v>
       </c>
-      <c r="M3">
-        <v>0</v>
-      </c>
-      <c r="N3">
+      <c r="M3" s="0">
+        <v>0</v>
+      </c>
+      <c r="N3" s="0">
         <v>1.2540430987612916</v>
       </c>
-      <c r="O3">
+      <c r="O3" s="0">
         <v>4.017047509867183</v>
       </c>
-      <c r="P3">
+      <c r="P3" s="0">
         <v>0.88016368853402249</v>
       </c>
-      <c r="Q3">
+      <c r="Q3" s="0">
         <v>0.24947670056123128</v>
       </c>
-      <c r="R3">
+      <c r="R3" s="0">
         <v>15.041820726873913</v>
       </c>
-      <c r="S3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="S3" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.25">
+      <c r="A4" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="B4">
-        <v>32</v>
-      </c>
-      <c r="C4">
+      <c r="B4" s="0">
+        <v>32</v>
+      </c>
+      <c r="C4" s="0">
         <v>200</v>
       </c>
-      <c r="D4">
-        <v>214.7</v>
-      </c>
-      <c r="E4">
+      <c r="D4" s="0">
+        <v>214.69999999999999</v>
+      </c>
+      <c r="E4" s="0">
         <v>14.803564999999999</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="0">
         <v>1.1868000000000001</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="0">
         <v>198.48110236220467</v>
       </c>
-      <c r="I4">
+      <c r="I4" s="0">
         <v>4.7204035433070866</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="0">
         <v>10.937511631836504</v>
       </c>
-      <c r="K4">
+      <c r="K4" s="0">
         <v>31.560103796200337</v>
       </c>
-      <c r="L4">
+      <c r="L4" s="0">
         <v>87.225196850393743</v>
       </c>
-      <c r="M4">
-        <v>0</v>
-      </c>
-      <c r="N4">
+      <c r="M4" s="0">
+        <v>0</v>
+      </c>
+      <c r="N4" s="0">
         <v>2.6734156708533678</v>
       </c>
-      <c r="O4">
+      <c r="O4" s="0">
         <v>3.590153841841623</v>
       </c>
-      <c r="P4">
+      <c r="P4" s="0">
         <v>2.7950547935498253</v>
       </c>
-      <c r="Q4">
+      <c r="Q4" s="0">
         <v>0.76527408198974711</v>
       </c>
-      <c r="R4">
+      <c r="R4" s="0">
         <v>11.591133782860224</v>
       </c>
-      <c r="S4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="S4" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.25">
+      <c r="A5" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="B5">
-        <v>32</v>
-      </c>
-      <c r="C5">
+      <c r="B5" s="0">
+        <v>32</v>
+      </c>
+      <c r="C5" s="0">
         <v>500</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="0">
         <v>514.70000000000005</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="0">
         <v>35.488565000000001</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="0">
         <v>2.7519999999999998</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="0">
         <v>501.79519230769228</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="0">
         <v>5.1345235576923081</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="0">
         <v>17.324857176970109</v>
       </c>
-      <c r="K5">
+      <c r="K5" s="0">
         <v>30.669425990489138</v>
       </c>
-      <c r="L5">
+      <c r="L5" s="0">
         <v>89.622115384615398</v>
       </c>
-      <c r="M5">
-        <v>0</v>
-      </c>
-      <c r="N5">
+      <c r="M5" s="0">
+        <v>0</v>
+      </c>
+      <c r="N5" s="0">
         <v>1.5959719712098357</v>
       </c>
-      <c r="O5">
+      <c r="O5" s="0">
         <v>3.7866055202723881</v>
       </c>
-      <c r="P5">
+      <c r="P5" s="0">
         <v>3.4262658647685331</v>
       </c>
-      <c r="Q5">
+      <c r="Q5" s="0">
         <v>0.89640242518304558</v>
       </c>
-      <c r="R5">
-        <v>4.6013505199247573E-2</v>
-      </c>
-      <c r="S5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="R5" s="0">
+        <v>0.046013505199247573</v>
+      </c>
+      <c r="S5" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.25">
+      <c r="A6" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="B6">
-        <v>32</v>
-      </c>
-      <c r="C6">
+      <c r="B6" s="0">
+        <v>32</v>
+      </c>
+      <c r="C6" s="0">
         <v>900</v>
       </c>
-      <c r="D6">
-        <v>914.7</v>
-      </c>
-      <c r="E6">
+      <c r="D6" s="0">
+        <v>914.70000000000005</v>
+      </c>
+      <c r="E6" s="0">
         <v>63.068565</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="0">
         <v>4.9062000000000001</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="0">
         <v>905.67198067632842</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="0">
         <v>5.4202536231884046</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="0">
         <v>23.36627758983288</v>
       </c>
-      <c r="K6">
+      <c r="K6" s="0">
         <v>29.996156779944307</v>
       </c>
-      <c r="L6">
+      <c r="L6" s="0">
         <v>89.785990338164169</v>
       </c>
-      <c r="M6">
-        <v>0</v>
-      </c>
-      <c r="N6">
+      <c r="M6" s="0">
+        <v>0</v>
+      </c>
+      <c r="N6" s="0">
         <v>2.1365264068116274</v>
       </c>
-      <c r="O6">
+      <c r="O6" s="0">
         <v>3.8782227988160041</v>
       </c>
-      <c r="P6">
+      <c r="P6" s="0">
         <v>3.1843633447634039</v>
       </c>
-      <c r="Q6">
+      <c r="Q6" s="0">
         <v>0.87890913316876806</v>
       </c>
-      <c r="R6">
-        <v>9.7277802092679E-2</v>
-      </c>
-      <c r="S6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="R6" s="0">
+        <v>0.097277802092679</v>
+      </c>
+      <c r="S6" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.25">
+      <c r="A7" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="B7">
-        <v>32</v>
-      </c>
-      <c r="C7">
+      <c r="B7" s="0">
+        <v>32</v>
+      </c>
+      <c r="C7" s="0">
         <v>1500</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="0">
         <v>1514.7</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="0">
         <v>104.438565</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="0">
         <v>7.9736000000000002</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="0">
         <v>1512.2045000000001</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="0">
         <v>5.6953334999999994</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="0">
         <v>30.602549671333804</v>
       </c>
-      <c r="K7">
+      <c r="K7" s="0">
         <v>29.434455296241719</v>
       </c>
-      <c r="L7">
+      <c r="L7" s="0">
         <v>84.637999999999991</v>
       </c>
-      <c r="M7">
-        <v>0</v>
-      </c>
-      <c r="N7">
+      <c r="M7" s="0">
+        <v>0</v>
+      </c>
+      <c r="N7" s="0">
         <v>1.5706253755596031</v>
       </c>
-      <c r="O7">
+      <c r="O7" s="0">
         <v>3.8441632097432428</v>
       </c>
-      <c r="P7">
+      <c r="P7" s="0">
         <v>2.084925107636002</v>
       </c>
-      <c r="Q7">
+      <c r="Q7" s="0">
         <v>0.68103295133502428</v>
       </c>
-      <c r="R7">
+      <c r="R7" s="0">
         <v>19.5469118999427</v>
       </c>
-      <c r="S7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="S7" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.25">
+      <c r="A8" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="B8">
-        <v>32</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="D8">
-        <v>14.7</v>
-      </c>
-      <c r="E8">
+      <c r="B8" s="0">
+        <v>32</v>
+      </c>
+      <c r="C8" s="0">
+        <v>0</v>
+      </c>
+      <c r="D8" s="0">
+        <v>14.699999999999999</v>
+      </c>
+      <c r="E8" s="0">
         <v>1.0135649999999998</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="0">
         <v>0.15759999999999999</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="H8">
-        <v>3.4589800443458975E-2</v>
-      </c>
-      <c r="I8">
+      <c r="H8" s="0">
+        <v>0.034589800443458975</v>
+      </c>
+      <c r="I8" s="0">
         <v>5.1274099778270523</v>
       </c>
-      <c r="J8">
+      <c r="J8" s="0">
         <v>5.0409025147510187</v>
       </c>
-      <c r="K8">
+      <c r="K8" s="0">
         <v>33.289447874412751</v>
       </c>
-      <c r="L8">
+      <c r="L8" s="0">
         <v>99.925498891352575</v>
       </c>
-      <c r="M8">
-        <v>0</v>
-      </c>
-      <c r="N8">
+      <c r="M8" s="0">
+        <v>0</v>
+      </c>
+      <c r="N8" s="0">
         <v>1.2197271089269492</v>
       </c>
-      <c r="O8">
+      <c r="O8" s="0">
         <v>3.8849882239618729</v>
       </c>
-      <c r="P8">
+      <c r="P8" s="0">
         <v>0.95988049606448755</v>
       </c>
-      <c r="Q8">
+      <c r="Q8" s="0">
         <v>0.28651369875411425</v>
       </c>
-      <c r="R8">
-        <v>9.6801776262924757E-2</v>
-      </c>
-      <c r="S8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="R8" s="0">
+        <v>0.096801776262924757</v>
+      </c>
+      <c r="S8" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.25">
+      <c r="A9" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="B9">
-        <v>32</v>
-      </c>
-      <c r="C9">
+      <c r="B9" s="0">
+        <v>32</v>
+      </c>
+      <c r="C9" s="0">
         <v>50</v>
       </c>
-      <c r="D9">
-        <v>64.7</v>
-      </c>
-      <c r="E9">
+      <c r="D9" s="0">
+        <v>64.700000000000003</v>
+      </c>
+      <c r="E9" s="0">
         <v>4.4610649999999996</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="0">
         <v>0.63029999999999997</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="0">
         <v>47.250891632373126</v>
       </c>
-      <c r="I9">
+      <c r="I9" s="0">
         <v>3.9248589849108382</v>
       </c>
-      <c r="J9">
+      <c r="J9" s="0">
         <v>5.6614757753759042</v>
       </c>
-      <c r="K9">
+      <c r="K9" s="0">
         <v>33.08237160652218</v>
       </c>
-      <c r="L9">
+      <c r="L9" s="0">
         <v>99.315912208504798</v>
       </c>
-      <c r="M9">
-        <v>0</v>
-      </c>
-      <c r="N9">
+      <c r="M9" s="0">
+        <v>0</v>
+      </c>
+      <c r="N9" s="0">
         <v>1.7724470576103351</v>
       </c>
-      <c r="O9">
+      <c r="O9" s="0">
         <v>3.5910982686787105</v>
       </c>
-      <c r="P9">
+      <c r="P9" s="0">
         <v>1.1295391952443583</v>
       </c>
-      <c r="Q9">
+      <c r="Q9" s="0">
         <v>0.33772752182948429</v>
       </c>
-      <c r="R9">
+      <c r="R9" s="0">
         <v>3.2072281471523798</v>
       </c>
-      <c r="S9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="S9" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.25">
+      <c r="A10" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="B10">
-        <v>32</v>
-      </c>
-      <c r="C10">
+      <c r="B10" s="0">
+        <v>32</v>
+      </c>
+      <c r="C10" s="0">
         <v>200</v>
       </c>
-      <c r="D10">
-        <v>214.7</v>
-      </c>
-      <c r="E10">
+      <c r="D10" s="0">
+        <v>214.69999999999999</v>
+      </c>
+      <c r="E10" s="0">
         <v>14.803564999999999</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="0">
         <v>2.3591000000000002</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="0">
         <v>196.90300230946883</v>
       </c>
-      <c r="I10">
+      <c r="I10" s="0">
         <v>3.4341660508083156</v>
       </c>
-      <c r="J10">
+      <c r="J10" s="0">
         <v>8.8750112185295063</v>
       </c>
-      <c r="K10">
+      <c r="K10" s="0">
         <v>32.201180555555545</v>
       </c>
-      <c r="L10">
+      <c r="L10" s="0">
         <v>100</v>
       </c>
-      <c r="M10">
-        <v>0</v>
-      </c>
-      <c r="N10">
+      <c r="M10" s="0">
+        <v>0</v>
+      </c>
+      <c r="N10" s="0">
         <v>2.2423254386194347</v>
       </c>
-      <c r="O10">
+      <c r="O10" s="0">
         <v>3.2283086787301234</v>
       </c>
-      <c r="P10">
+      <c r="P10" s="0">
         <v>2.6572777636791054</v>
       </c>
-      <c r="Q10">
+      <c r="Q10" s="0">
         <v>0.72962676422545669</v>
       </c>
-      <c r="R10">
-        <v>0</v>
-      </c>
-      <c r="S10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="R10" s="0">
+        <v>0</v>
+      </c>
+      <c r="S10" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.25">
+      <c r="A11" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="B11">
-        <v>32</v>
-      </c>
-      <c r="C11">
+      <c r="B11" s="0">
+        <v>32</v>
+      </c>
+      <c r="C11" s="0">
         <v>500</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="0">
         <v>514.70000000000005</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="0">
         <v>35.488565000000001</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="0">
         <v>5.4836</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="0">
         <v>498.9257918552035</v>
       </c>
-      <c r="I11">
+      <c r="I11" s="0">
         <v>4.9094751131221717</v>
       </c>
-      <c r="J11">
+      <c r="J11" s="0">
         <v>15.248373578269492</v>
       </c>
-      <c r="K11">
+      <c r="K11" s="0">
         <v>30.789832946499335</v>
       </c>
-      <c r="L11">
+      <c r="L11" s="0">
         <v>100</v>
       </c>
-      <c r="M11">
-        <v>0</v>
-      </c>
-      <c r="N11">
+      <c r="M11" s="0">
+        <v>0</v>
+      </c>
+      <c r="N11" s="0">
         <v>1.1155165668981717</v>
       </c>
-      <c r="O11">
+      <c r="O11" s="0">
         <v>3.5149867191738773</v>
       </c>
-      <c r="P11">
+      <c r="P11" s="0">
         <v>3.2093746591529744</v>
       </c>
-      <c r="Q11">
+      <c r="Q11" s="0">
         <v>0.84924061944480778</v>
       </c>
-      <c r="R11">
-        <v>0</v>
-      </c>
-      <c r="S11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="R11" s="0">
+        <v>0</v>
+      </c>
+      <c r="S11" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.25">
+      <c r="A12" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="B12">
-        <v>32</v>
-      </c>
-      <c r="C12">
+      <c r="B12" s="0">
+        <v>32</v>
+      </c>
+      <c r="C12" s="0">
         <v>900</v>
       </c>
-      <c r="D12">
-        <v>914.7</v>
-      </c>
-      <c r="E12">
+      <c r="D12" s="0">
+        <v>914.70000000000005</v>
+      </c>
+      <c r="E12" s="0">
         <v>63.068565</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="0">
         <v>9.8087</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="0">
         <v>902.25786163522014</v>
       </c>
-      <c r="I12">
+      <c r="I12" s="0">
         <v>5.2859710691823905</v>
       </c>
-      <c r="J12">
+      <c r="J12" s="0">
         <v>19.136441189911682</v>
       </c>
-      <c r="K12">
+      <c r="K12" s="0">
         <v>30.023145309623416</v>
       </c>
-      <c r="L12">
+      <c r="L12" s="0">
         <v>98.389622641509433</v>
       </c>
-      <c r="M12">
-        <v>0</v>
-      </c>
-      <c r="N12">
+      <c r="M12" s="0">
+        <v>0</v>
+      </c>
+      <c r="N12" s="0">
         <v>1.864304697744283</v>
       </c>
-      <c r="O12">
+      <c r="O12" s="0">
         <v>3.643698563357221</v>
       </c>
-      <c r="P12">
+      <c r="P12" s="0">
         <v>2.6377785667324614</v>
       </c>
-      <c r="Q12">
+      <c r="Q12" s="0">
         <v>0.77204972065196631</v>
       </c>
-      <c r="R12">
+      <c r="R12" s="0">
         <v>11.755583377746854</v>
       </c>
-      <c r="S12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="S12" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.25">
+      <c r="A13" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="B13">
-        <v>32</v>
-      </c>
-      <c r="C13">
+      <c r="B13" s="0">
+        <v>32</v>
+      </c>
+      <c r="C13" s="0">
         <v>1500</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="0">
         <v>1514.7</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="0">
         <v>104.438565</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="0">
         <v>16.0169</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="H13">
+      <c r="H13" s="0">
         <v>1509.8943019943017</v>
       </c>
-      <c r="I13">
+      <c r="I13" s="0">
         <v>4.8871396011396007</v>
       </c>
-      <c r="J13">
+      <c r="J13" s="0">
         <v>22.583947249796918</v>
       </c>
-      <c r="K13">
+      <c r="K13" s="0">
         <v>29.553734050771727</v>
       </c>
-      <c r="L13">
+      <c r="L13" s="0">
         <v>100</v>
       </c>
-      <c r="M13">
-        <v>0</v>
-      </c>
-      <c r="N13">
+      <c r="M13" s="0">
+        <v>0</v>
+      </c>
+      <c r="N13" s="0">
         <v>2.6680697163672491</v>
       </c>
-      <c r="O13">
+      <c r="O13" s="0">
         <v>3.5195640903707481</v>
       </c>
-      <c r="P13">
+      <c r="P13" s="0">
         <v>2.0371158532082272</v>
       </c>
-      <c r="Q13">
+      <c r="Q13" s="0">
         <v>0.73937305865185432</v>
       </c>
-      <c r="R13">
-        <v>0</v>
-      </c>
-      <c r="S13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="R13" s="0">
+        <v>0</v>
+      </c>
+      <c r="S13" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.25">
+      <c r="A14" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="B14">
-        <v>32</v>
-      </c>
-      <c r="C14">
-        <v>0</v>
-      </c>
-      <c r="D14">
-        <v>14.7</v>
-      </c>
-      <c r="E14">
+      <c r="B14" s="0">
+        <v>32</v>
+      </c>
+      <c r="C14" s="0">
+        <v>0</v>
+      </c>
+      <c r="D14" s="0">
+        <v>14.699999999999999</v>
+      </c>
+      <c r="E14" s="0">
         <v>1.0135649999999998</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="0">
         <v>1.7436</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G14" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="H14">
+      <c r="H14" s="0">
         <v>1.1364341085271319</v>
       </c>
-      <c r="I14">
+      <c r="I14" s="0">
         <v>19.97357906976745</v>
       </c>
-      <c r="J14">
+      <c r="J14" s="0">
         <v>7.7575418333068953</v>
       </c>
-      <c r="K14">
+      <c r="K14" s="0">
         <v>31.247848865186349</v>
       </c>
-      <c r="L14">
-        <v>0</v>
-      </c>
-      <c r="M14">
+      <c r="L14" s="0">
+        <v>0</v>
+      </c>
+      <c r="M14" s="0">
         <v>100</v>
       </c>
-      <c r="N14">
+      <c r="N14" s="0">
         <v>2.4263110227127149</v>
       </c>
-      <c r="O14">
+      <c r="O14" s="0">
         <v>33.022844824569816</v>
       </c>
-      <c r="P14">
+      <c r="P14" s="0">
         <v>0.59129778243089126</v>
       </c>
-      <c r="Q14">
+      <c r="Q14" s="0">
         <v>0.42843052533663623</v>
       </c>
-      <c r="R14">
-        <v>0</v>
-      </c>
-      <c r="S14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="R14" s="0">
+        <v>0</v>
+      </c>
+      <c r="S14" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.25">
+      <c r="A15" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="B15">
-        <v>32</v>
-      </c>
-      <c r="C15">
+      <c r="B15" s="0">
+        <v>32</v>
+      </c>
+      <c r="C15" s="0">
         <v>50</v>
       </c>
-      <c r="D15">
-        <v>64.7</v>
-      </c>
-      <c r="E15">
+      <c r="D15" s="0">
+        <v>64.700000000000003</v>
+      </c>
+      <c r="E15" s="0">
         <v>4.4610649999999996</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="0">
         <v>7.0845000000000002</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="H15">
+      <c r="H15" s="0">
         <v>48.184444444444445</v>
       </c>
-      <c r="I15">
+      <c r="I15" s="0">
         <v>4.5322257777777768</v>
       </c>
-      <c r="J15">
+      <c r="J15" s="0">
         <v>15.324929975443389</v>
       </c>
-      <c r="K15">
+      <c r="K15" s="0">
         <v>31.865021680763984</v>
       </c>
-      <c r="L15">
-        <v>0</v>
-      </c>
-      <c r="M15">
+      <c r="L15" s="0">
+        <v>0</v>
+      </c>
+      <c r="M15" s="0">
         <v>100</v>
       </c>
-      <c r="N15">
+      <c r="N15" s="0">
         <v>0.33337797320139995</v>
       </c>
-      <c r="O15">
+      <c r="O15" s="0">
         <v>3.6738301317941975</v>
       </c>
-      <c r="P15">
+      <c r="P15" s="0">
         <v>0.80639047384132334</v>
       </c>
-      <c r="Q15">
+      <c r="Q15" s="0">
         <v>0.29632443275269749</v>
       </c>
-      <c r="R15">
-        <v>0</v>
-      </c>
-      <c r="S15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="R15" s="0">
+        <v>0</v>
+      </c>
+      <c r="S15" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.25">
+      <c r="A16" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="B16">
-        <v>32</v>
-      </c>
-      <c r="C16">
+      <c r="B16" s="0">
+        <v>32</v>
+      </c>
+      <c r="C16" s="0">
         <v>200</v>
       </c>
-      <c r="D16">
-        <v>214.7</v>
-      </c>
-      <c r="E16">
+      <c r="D16" s="0">
+        <v>214.69999999999999</v>
+      </c>
+      <c r="E16" s="0">
         <v>14.803564999999999</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="0">
         <v>28.2637</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G16" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="H16">
+      <c r="H16" s="0">
         <v>197.60777202072532</v>
       </c>
-      <c r="I16">
+      <c r="I16" s="0">
         <v>3.927444041450777</v>
       </c>
-      <c r="J16">
+      <c r="J16" s="0">
         <v>37.162242071599039</v>
       </c>
-      <c r="K16">
+      <c r="K16" s="0">
         <v>30.835474119331728</v>
       </c>
-      <c r="L16">
-        <v>0</v>
-      </c>
-      <c r="M16">
+      <c r="L16" s="0">
+        <v>0</v>
+      </c>
+      <c r="M16" s="0">
         <v>99.898963730569946</v>
       </c>
-      <c r="N16">
+      <c r="N16" s="0">
         <v>0.85871252334803438</v>
       </c>
-      <c r="O16">
+      <c r="O16" s="0">
         <v>3.1448903477470145</v>
       </c>
-      <c r="P16">
+      <c r="P16" s="0">
         <v>0.54138861450113618</v>
       </c>
-      <c r="Q16">
+      <c r="Q16" s="0">
         <v>0.22602155329980328</v>
       </c>
-      <c r="R16">
-        <v>0</v>
-      </c>
-      <c r="S16">
+      <c r="R16" s="0">
+        <v>0</v>
+      </c>
+      <c r="S16" s="0">
         <v>0.6685641982781797</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.25">
+      <c r="A17" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="B17">
-        <v>32</v>
-      </c>
-      <c r="C17">
+      <c r="B17" s="0">
+        <v>32</v>
+      </c>
+      <c r="C17" s="0">
         <v>500</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="0">
         <v>514.70000000000005</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="0">
         <v>35.488565000000001</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="0">
         <v>75.694199999999995</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="H17">
+      <c r="H17" s="0">
         <v>504.57743055555574</v>
       </c>
-      <c r="I17">
+      <c r="I17" s="0">
         <v>3.670116666666666</v>
       </c>
-      <c r="J17">
+      <c r="J17" s="0">
         <v>87.394100698133371</v>
       </c>
-      <c r="K17">
+      <c r="K17" s="0">
         <v>31.789277421866643</v>
       </c>
-      <c r="L17">
-        <v>0</v>
-      </c>
-      <c r="M17">
+      <c r="L17" s="0">
+        <v>0</v>
+      </c>
+      <c r="M17" s="0">
         <v>72.320486111111109</v>
       </c>
-      <c r="N17">
+      <c r="N17" s="0">
         <v>3.1733885309996048</v>
       </c>
-      <c r="O17">
+      <c r="O17" s="0">
         <v>3.6318289864035225</v>
       </c>
-      <c r="P17">
+      <c r="P17" s="0">
         <v>0.63934096509314597</v>
       </c>
-      <c r="Q17">
+      <c r="Q17" s="0">
         <v>0.1587645698654859</v>
       </c>
-      <c r="R17">
-        <v>0</v>
-      </c>
-      <c r="S17">
+      <c r="R17" s="0">
+        <v>0</v>
+      </c>
+      <c r="S17" s="0">
         <v>44.563462523656831</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.25">
+      <c r="A18" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="B18">
-        <v>32</v>
-      </c>
-      <c r="C18">
+      <c r="B18" s="0">
+        <v>32</v>
+      </c>
+      <c r="C18" s="0">
         <v>900</v>
       </c>
-      <c r="D18">
-        <v>914.7</v>
-      </c>
-      <c r="E18">
+      <c r="D18" s="0">
+        <v>914.70000000000005</v>
+      </c>
+      <c r="E18" s="0">
         <v>63.068565</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="0">
         <v>188.47470000000001</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G18" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="H18">
+      <c r="H18" s="0">
         <v>907.42638888888905</v>
       </c>
-      <c r="I18">
+      <c r="I18" s="0">
         <v>3.5231287037037031</v>
       </c>
-      <c r="J18">
+      <c r="J18" s="0">
         <v>204.04287756218898</v>
       </c>
-      <c r="K18">
+      <c r="K18" s="0">
         <v>30.784062602700786</v>
       </c>
-      <c r="L18">
-        <v>0</v>
-      </c>
-      <c r="M18">
+      <c r="L18" s="0">
+        <v>0</v>
+      </c>
+      <c r="M18" s="0">
         <v>98.418981481481481</v>
       </c>
-      <c r="N18">
+      <c r="N18" s="0">
         <v>1.9176773540167058</v>
       </c>
-      <c r="O18">
+      <c r="O18" s="0">
         <v>3.4626444082333871</v>
       </c>
-      <c r="P18">
+      <c r="P18" s="0">
         <v>2.4034296757844804</v>
       </c>
-      <c r="Q18">
+      <c r="Q18" s="0">
         <v>0.32864614436748485</v>
       </c>
-      <c r="R18">
-        <v>0</v>
-      </c>
-      <c r="S18">
+      <c r="R18" s="0">
+        <v>0</v>
+      </c>
+      <c r="S18" s="0">
         <v>10.581447603064511</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.25">
+      <c r="A19" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="B19">
-        <v>32</v>
-      </c>
-      <c r="C19">
+      <c r="B19" s="0">
+        <v>32</v>
+      </c>
+      <c r="C19" s="0">
         <v>1500</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="0">
         <v>1514.7</v>
       </c>
-      <c r="E19">
+      <c r="E19" s="0">
         <v>104.438565</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="0">
         <v>709.51559999999995</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G19" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="H19">
+      <c r="H19" s="0">
         <v>1510.1233962264148</v>
       </c>
-      <c r="I19">
+      <c r="I19" s="0">
         <v>2.8830139622641515</v>
       </c>
-      <c r="J19">
+      <c r="J19" s="0">
         <v>771.82309045112811</v>
       </c>
-      <c r="K19">
+      <c r="K19" s="0">
         <v>32.392472813186821</v>
       </c>
-      <c r="L19">
-        <v>0</v>
-      </c>
-      <c r="M19">
+      <c r="L19" s="0">
+        <v>0</v>
+      </c>
+      <c r="M19" s="0">
         <v>69.524150943396236</v>
       </c>
-      <c r="N19">
+      <c r="N19" s="0">
         <v>4.1855971223279846</v>
       </c>
-      <c r="O19">
+      <c r="O19" s="0">
         <v>2.9869330835744008</v>
       </c>
-      <c r="P19">
-        <v>5.0331221152869903</v>
-      </c>
-      <c r="Q19">
+      <c r="P19" s="0">
+        <v>5.0331221152869912</v>
+      </c>
+      <c r="Q19" s="0">
         <v>0.41331040641822658</v>
       </c>
-      <c r="R19">
-        <v>0</v>
-      </c>
-      <c r="S19">
+      <c r="R19" s="0">
+        <v>0</v>
+      </c>
+      <c r="S19" s="0">
         <v>43.733713221019087</v>
       </c>
     </row>

</xml_diff>

<commit_message>
results of main cal main pr and main data extract
</commit_message>
<xml_diff>
--- a/results/cal_250725_PR/calResults.xlsx
+++ b/results/cal_250725_PR/calResults.xlsx
@@ -1,26 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps/results/cal_250725_PR/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_1357E617CF19DF7F2B1B3B26FE012D16D10A0B41" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{018C2BF4-DA90-4078-BF9D-CC816F2F7758}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="1200" yWindow="1695" windowWidth="21600" windowHeight="11295"/>
+    <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0" fullCalcOnLoad="true"/>
+  <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="275" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="55" uniqueCount="24">
   <si>
     <t>Fluid</t>
   </si>
@@ -132,361 +125,36 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="0E2841"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="156082"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="E97132"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="196B24"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="A02B93"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="4EA72E"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="467886"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="96607D"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="true">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="false"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="true">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="false"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
-              <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:gradFill rotWithShape="true">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="false"/>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:S19"/>
-  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.5703125" customWidth="true"/>
     <col min="2" max="2" width="6.140625" customWidth="true"/>
     <col min="3" max="3" width="6.85546875" customWidth="true"/>
+    <col min="4" max="4" width="6.85546875" customWidth="true"/>
     <col min="5" max="5" width="10.7109375" customWidth="true"/>
     <col min="6" max="6" width="8.7109375" customWidth="true"/>
     <col min="7" max="7" width="12" customWidth="true"/>
     <col min="8" max="8" width="13.7109375" customWidth="true"/>
     <col min="9" max="9" width="11.7109375" customWidth="true"/>
+    <col min="10" max="10" width="11.7109375" customWidth="true"/>
+    <col min="11" max="11" width="11.7109375" customWidth="true"/>
     <col min="12" max="12" width="15" customWidth="true"/>
+    <col min="13" max="13" width="15" customWidth="true"/>
     <col min="14" max="14" width="12.7109375" customWidth="true"/>
     <col min="15" max="15" width="11.7109375" customWidth="true"/>
     <col min="16" max="16" width="12.7109375" customWidth="true"/>
+    <col min="17" max="17" width="12.7109375" customWidth="true"/>
     <col min="18" max="18" width="13.7109375" customWidth="true"/>
     <col min="19" max="19" width="12.7109375" customWidth="true"/>
-    <col min="4" max="4" width="6.85546875" customWidth="true"/>
-    <col min="10" max="10" width="11.7109375" customWidth="true"/>
-    <col min="11" max="11" width="11.7109375" customWidth="true"/>
-    <col min="13" max="13" width="15" customWidth="true"/>
-    <col min="17" max="17" width="12.7109375" customWidth="true"/>
   </cols>
   <sheetData>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
@@ -545,7 +213,7 @@
         <v>23</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2" s="0" t="s">
         <v>1</v>
       </c>
@@ -604,7 +272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.25">
+    <row r="3">
       <c r="A3" s="0" t="s">
         <v>1</v>
       </c>
@@ -663,7 +331,7 @@
         <v>0</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.25">
+    <row r="4">
       <c r="A4" s="0" t="s">
         <v>1</v>
       </c>
@@ -722,7 +390,7 @@
         <v>0</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.25">
+    <row r="5">
       <c r="A5" s="0" t="s">
         <v>1</v>
       </c>
@@ -781,7 +449,7 @@
         <v>0</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.25">
+    <row r="6">
       <c r="A6" s="0" t="s">
         <v>1</v>
       </c>
@@ -840,7 +508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.25">
+    <row r="7">
       <c r="A7" s="0" t="s">
         <v>1</v>
       </c>
@@ -899,7 +567,7 @@
         <v>0</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.25">
+    <row r="8">
       <c r="A8" s="0" t="s">
         <v>2</v>
       </c>
@@ -958,7 +626,7 @@
         <v>0</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.25">
+    <row r="9">
       <c r="A9" s="0" t="s">
         <v>2</v>
       </c>
@@ -1017,7 +685,7 @@
         <v>0</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.25">
+    <row r="10">
       <c r="A10" s="0" t="s">
         <v>2</v>
       </c>
@@ -1076,7 +744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.25">
+    <row r="11">
       <c r="A11" s="0" t="s">
         <v>2</v>
       </c>
@@ -1135,7 +803,7 @@
         <v>0</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.25">
+    <row r="12">
       <c r="A12" s="0" t="s">
         <v>2</v>
       </c>
@@ -1194,7 +862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.25">
+    <row r="13">
       <c r="A13" s="0" t="s">
         <v>2</v>
       </c>
@@ -1253,7 +921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.25">
+    <row r="14">
       <c r="A14" s="0" t="s">
         <v>3</v>
       </c>
@@ -1312,7 +980,7 @@
         <v>0</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.25">
+    <row r="15">
       <c r="A15" s="0" t="s">
         <v>3</v>
       </c>
@@ -1371,7 +1039,7 @@
         <v>0</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.25">
+    <row r="16">
       <c r="A16" s="0" t="s">
         <v>3</v>
       </c>
@@ -1430,7 +1098,7 @@
         <v>0.6685641982781797</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.25">
+    <row r="17">
       <c r="A17" s="0" t="s">
         <v>3</v>
       </c>
@@ -1489,7 +1157,7 @@
         <v>44.563462523656831</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.25">
+    <row r="18">
       <c r="A18" s="0" t="s">
         <v>3</v>
       </c>
@@ -1548,7 +1216,7 @@
         <v>10.581447603064511</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.25">
+    <row r="19">
       <c r="A19" s="0" t="s">
         <v>3</v>
       </c>
@@ -1608,6 +1276,5 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Commenting on calDataQAll, before removing
</commit_message>
<xml_diff>
--- a/results/cal_250725_PR/calResults.xlsx
+++ b/results/cal_250725_PR/calResults.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="366" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="368" uniqueCount="173">
   <si>
     <t>Fluid</t>
   </si>
@@ -85,6 +85,447 @@
     <t>Z_ref</t>
   </si>
   <si>
+    <t>fluid_ref</t>
+  </si>
+  <si>
+    <t>T_ref</t>
+  </si>
+  <si>
+    <t>Ppsig_ref</t>
+  </si>
+  <si>
+    <t>st</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:35:22.000, 07/29/2025 15:35:33.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:32:17.000, 07/29/2025 15:32:50.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:34:33.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:42:58.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:42:10.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:41:20.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:39:28.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:45:08.000, 07/29/2025 15:49:47.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:48:41.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:47:41.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:46:06.000, 07/29/2025 15:46:54.000, 07/29/2025 15:50:50.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:54:51.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:53:59.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:53:19.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:51:53.000, 07/29/2025 15:55:35.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:00:08.000, 07/29/2025 16:01:24.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:59:29.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:58:50.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:57:04.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:05:18.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:04:38.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:03:58.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:02:22.000, 07/29/2025 16:03:09.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:10:13.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 13:52:02.000, 07/29/2025 13:57:24.000, 07/29/2025 14:01:02.000, 07/29/2025 14:01:08.000, 07/29/2025 14:01:11.000, 07/29/2025 14:01:19.000, 07/29/2025 14:13:14.000, 07/29/2025 14:14:08.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:01:54.000, 07/29/2025 14:02:06.000, 07/29/2025 14:02:09.000, 07/29/2025 14:02:12.000, 07/29/2025 14:02:17.000, 07/29/2025 14:02:21.000, 07/29/2025 14:02:27.000, 07/29/2025 14:02:32.000, 07/29/2025 14:02:34.000, 07/29/2025 14:02:39.000, 07/29/2025 14:02:44.000, 07/29/2025 14:02:48.000, 07/29/2025 14:02:55.000, 07/29/2025 14:02:58.000, 07/29/2025 14:03:01.000, 07/29/2025 14:03:05.000, 07/29/2025 14:03:13.000, 07/29/2025 14:03:16.000, 07/29/2025 14:03:20.000, 07/29/2025 14:03:25.000, 07/29/2025 14:03:31.000, 07/29/2025 14:03:34.000, 07/29/2025 14:03:40.000, 07/29/2025 14:03:48.000, 07/29/2025 14:03:55.000, 07/29/2025 14:04:13.000, 07/29/2025 14:04:19.000, 07/29/2025 14:04:25.000, 07/29/2025 14:04:27.000, 07/29/2025 14:04:36.000, 07/29/2025 14:04:43.000, 07/29/2025 14:04:50.000, 07/29/2025 14:04:58.000, 07/29/2025 14:05:16.000, 07/29/2025 14:05:18.000, 07/29/2025 14:05:34.000, 07/29/2025 14:05:46.000, 07/29/2025 14:06:09.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:09:00.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:25:26.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:16:41.000, 07/29/2025 14:16:54.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:21:06.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:22:33.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:35:29.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:33:54.000, 07/29/2025 14:37:45.000, 07/29/2025 14:39:47.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:31:43.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:36:39.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:45:16.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:44:26.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:42:16.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:46:01.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:53:42.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:52:45.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:51:17.000, 07/29/2025 14:51:28.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:49:01.000, 07/29/2025 14:54:49.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:01:27.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:00:39.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:58:46.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:56:33.000, 07/29/2025 14:57:31.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:23:07.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:25:23.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:26:05.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:26:52.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:21:19.000, 07/29/2025 16:40:37.000, 07/29/2025 16:44:25.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:41:50.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:42:35.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:43:24.000, 07/29/2025 16:45:05.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:20:25.000, 07/29/2025 16:34:59.000, 07/29/2025 16:38:59.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:36:21.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:37:25.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:38:16.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:19:04.000, 07/29/2025 16:33:16.000, 07/29/2025 16:56:33.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:59:35.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 17:00:19.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 17:00:57.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:46:40.000, 07/29/2025 16:47:27.000, 07/29/2025 16:50:32.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:47:22.000, 07/29/2025 16:48:45.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:47:15.000, 07/29/2025 16:49:19.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:46:58.000, 07/29/2025 16:49:50.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 17:07:54.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 17:07:52.000, 07/29/2025 17:09:39.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 17:07:47.000, 07/29/2025 17:10:59.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 17:07:38.000</t>
+  </si>
+  <si>
+    <t>et</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:35:28.000, 07/29/2025 15:35:35.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:32:45.000, 07/29/2025 15:32:50.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:35:21.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:44:47.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:42:57.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:42:09.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:41:19.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:45:08.000, 07/29/2025 15:50:49.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:49:46.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:48:40.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:46:52.000, 07/29/2025 15:47:40.000, 07/29/2025 15:51:07.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:55:34.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:54:50.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:53:58.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:53:18.000, 07/29/2025 15:55:56.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:01:12.000, 07/29/2025 16:01:25.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:00:07.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:59:28.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:58:49.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:05:50.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:05:17.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:04:37.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:03:07.000, 07/29/2025 16:03:56.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:13:13.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 13:52:05.000, 07/29/2025 14:01:00.000, 07/29/2025 14:01:06.000, 07/29/2025 14:01:09.000, 07/29/2025 14:01:12.000, 07/29/2025 14:01:19.000, 07/29/2025 14:13:21.000, 07/29/2025 14:14:09.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:02:04.000, 07/29/2025 14:02:06.000, 07/29/2025 14:02:10.000, 07/29/2025 14:02:14.000, 07/29/2025 14:02:19.000, 07/29/2025 14:02:25.000, 07/29/2025 14:02:27.000, 07/29/2025 14:02:32.000, 07/29/2025 14:02:36.000, 07/29/2025 14:02:42.000, 07/29/2025 14:02:46.000, 07/29/2025 14:02:52.000, 07/29/2025 14:02:55.000, 07/29/2025 14:02:59.000, 07/29/2025 14:03:03.000, 07/29/2025 14:03:10.000, 07/29/2025 14:03:14.000, 07/29/2025 14:03:18.000, 07/29/2025 14:03:23.000, 07/29/2025 14:03:29.000, 07/29/2025 14:03:32.000, 07/29/2025 14:03:38.000, 07/29/2025 14:03:46.000, 07/29/2025 14:03:53.000, 07/29/2025 14:03:58.000, 07/29/2025 14:04:14.000, 07/29/2025 14:04:20.000, 07/29/2025 14:04:25.000, 07/29/2025 14:04:29.000, 07/29/2025 14:04:36.000, 07/29/2025 14:04:43.000, 07/29/2025 14:04:51.000, 07/29/2025 14:05:00.000, 07/29/2025 14:05:16.000, 07/29/2025 14:05:18.000, 07/29/2025 14:05:34.000, 07/29/2025 14:06:05.000, 07/29/2025 14:06:11.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:09:03.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:25:33.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:16:41.000, 07/29/2025 14:21:05.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:22:32.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:25:24.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:36:38.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:35:28.000, 07/29/2025 14:38:30.000, 07/29/2025 14:39:48.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:33:53.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:37:44.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:46:00.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:45:15.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:44:25.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:47:29.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:54:48.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:53:41.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:51:26.000, 07/29/2025 14:52:44.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:51:16.000, 07/29/2025 14:55:13.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:03:00.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:01:26.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 15:00:38.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 14:57:29.000, 07/29/2025 14:58:45.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:25:22.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:26:04.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:26:51.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:28:54.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:21:23.000, 07/29/2025 16:41:49.000, 07/29/2025 16:45:04.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:42:34.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:43:22.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:44:24.000, 07/29/2025 16:45:05.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:20:29.000, 07/29/2025 16:36:20.000, 07/29/2025 16:39:16.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:37:24.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:38:15.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:38:58.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:19:19.000, 07/29/2025 16:33:33.000, 07/29/2025 16:59:34.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 17:00:18.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 17:00:56.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 17:02:00.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:46:57.000, 07/29/2025 16:48:44.000, 07/29/2025 16:50:58.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:47:26.000, 07/29/2025 16:49:18.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:47:21.000, 07/29/2025 16:49:49.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 16:47:14.000, 07/29/2025 16:50:31.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 17:09:38.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 17:07:53.000, 07/29/2025 17:10:58.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 17:07:51.000, 07/29/2025 17:12:00.000</t>
+  </si>
+  <si>
+    <t>07/29/2025 17:07:46.000</t>
+  </si>
+  <si>
     <t>phase_ref</t>
   </si>
   <si>
@@ -92,438 +533,6 @@
   </si>
   <si>
     <t>supercritical</t>
-  </si>
-  <si>
-    <t>st</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:35:22.000, 07/29/2025 15:35:33.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:32:17.000, 07/29/2025 15:32:50.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:34:33.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:42:58.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:42:10.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:41:20.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:39:28.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:45:08.000, 07/29/2025 15:49:47.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:48:41.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:47:41.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:46:06.000, 07/29/2025 15:46:54.000, 07/29/2025 15:50:50.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:54:51.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:53:59.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:53:19.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:51:53.000, 07/29/2025 15:55:35.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:00:08.000, 07/29/2025 16:01:24.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:59:29.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:58:50.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:57:04.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:05:18.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:04:38.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:03:58.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:02:22.000, 07/29/2025 16:03:09.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:10:13.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 13:52:02.000, 07/29/2025 13:57:24.000, 07/29/2025 14:01:02.000, 07/29/2025 14:01:08.000, 07/29/2025 14:01:11.000, 07/29/2025 14:01:19.000, 07/29/2025 14:13:14.000, 07/29/2025 14:14:08.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:01:54.000, 07/29/2025 14:02:06.000, 07/29/2025 14:02:09.000, 07/29/2025 14:02:12.000, 07/29/2025 14:02:17.000, 07/29/2025 14:02:21.000, 07/29/2025 14:02:27.000, 07/29/2025 14:02:32.000, 07/29/2025 14:02:34.000, 07/29/2025 14:02:39.000, 07/29/2025 14:02:44.000, 07/29/2025 14:02:48.000, 07/29/2025 14:02:55.000, 07/29/2025 14:02:58.000, 07/29/2025 14:03:01.000, 07/29/2025 14:03:05.000, 07/29/2025 14:03:13.000, 07/29/2025 14:03:16.000, 07/29/2025 14:03:20.000, 07/29/2025 14:03:25.000, 07/29/2025 14:03:31.000, 07/29/2025 14:03:34.000, 07/29/2025 14:03:40.000, 07/29/2025 14:03:48.000, 07/29/2025 14:03:55.000, 07/29/2025 14:04:13.000, 07/29/2025 14:04:19.000, 07/29/2025 14:04:25.000, 07/29/2025 14:04:27.000, 07/29/2025 14:04:36.000, 07/29/2025 14:04:43.000, 07/29/2025 14:04:50.000, 07/29/2025 14:04:58.000, 07/29/2025 14:05:16.000, 07/29/2025 14:05:18.000, 07/29/2025 14:05:34.000, 07/29/2025 14:05:46.000, 07/29/2025 14:06:09.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:09:00.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:25:26.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:16:41.000, 07/29/2025 14:16:54.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:21:06.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:22:33.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:35:29.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:33:54.000, 07/29/2025 14:37:45.000, 07/29/2025 14:39:47.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:31:43.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:36:39.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:45:16.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:44:26.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:42:16.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:46:01.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:53:42.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:52:45.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:51:17.000, 07/29/2025 14:51:28.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:49:01.000, 07/29/2025 14:54:49.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:01:27.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:00:39.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:58:46.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:56:33.000, 07/29/2025 14:57:31.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:23:07.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:25:23.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:26:05.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:26:52.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:21:19.000, 07/29/2025 16:40:37.000, 07/29/2025 16:44:25.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:41:50.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:42:35.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:43:24.000, 07/29/2025 16:45:05.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:20:25.000, 07/29/2025 16:34:59.000, 07/29/2025 16:38:59.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:36:21.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:37:25.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:38:16.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:19:04.000, 07/29/2025 16:33:16.000, 07/29/2025 16:56:33.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:59:35.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 17:00:19.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 17:00:57.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:46:40.000, 07/29/2025 16:47:27.000, 07/29/2025 16:50:32.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:47:22.000, 07/29/2025 16:48:45.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:47:15.000, 07/29/2025 16:49:19.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:46:58.000, 07/29/2025 16:49:50.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 17:07:54.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 17:07:52.000, 07/29/2025 17:09:39.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 17:07:47.000, 07/29/2025 17:10:59.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 17:07:38.000</t>
-  </si>
-  <si>
-    <t>et</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:35:28.000, 07/29/2025 15:35:35.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:32:45.000, 07/29/2025 15:32:50.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:35:21.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:44:47.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:42:57.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:42:09.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:41:19.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:45:08.000, 07/29/2025 15:50:49.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:49:46.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:48:40.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:46:52.000, 07/29/2025 15:47:40.000, 07/29/2025 15:51:07.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:55:34.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:54:50.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:53:58.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:53:18.000, 07/29/2025 15:55:56.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:01:12.000, 07/29/2025 16:01:25.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:00:07.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:59:28.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:58:49.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:05:50.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:05:17.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:04:37.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:03:07.000, 07/29/2025 16:03:56.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:13:13.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 13:52:05.000, 07/29/2025 14:01:00.000, 07/29/2025 14:01:06.000, 07/29/2025 14:01:09.000, 07/29/2025 14:01:12.000, 07/29/2025 14:01:19.000, 07/29/2025 14:13:21.000, 07/29/2025 14:14:09.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:02:04.000, 07/29/2025 14:02:06.000, 07/29/2025 14:02:10.000, 07/29/2025 14:02:14.000, 07/29/2025 14:02:19.000, 07/29/2025 14:02:25.000, 07/29/2025 14:02:27.000, 07/29/2025 14:02:32.000, 07/29/2025 14:02:36.000, 07/29/2025 14:02:42.000, 07/29/2025 14:02:46.000, 07/29/2025 14:02:52.000, 07/29/2025 14:02:55.000, 07/29/2025 14:02:59.000, 07/29/2025 14:03:03.000, 07/29/2025 14:03:10.000, 07/29/2025 14:03:14.000, 07/29/2025 14:03:18.000, 07/29/2025 14:03:23.000, 07/29/2025 14:03:29.000, 07/29/2025 14:03:32.000, 07/29/2025 14:03:38.000, 07/29/2025 14:03:46.000, 07/29/2025 14:03:53.000, 07/29/2025 14:03:58.000, 07/29/2025 14:04:14.000, 07/29/2025 14:04:20.000, 07/29/2025 14:04:25.000, 07/29/2025 14:04:29.000, 07/29/2025 14:04:36.000, 07/29/2025 14:04:43.000, 07/29/2025 14:04:51.000, 07/29/2025 14:05:00.000, 07/29/2025 14:05:16.000, 07/29/2025 14:05:18.000, 07/29/2025 14:05:34.000, 07/29/2025 14:06:05.000, 07/29/2025 14:06:11.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:09:03.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:25:33.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:16:41.000, 07/29/2025 14:21:05.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:22:32.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:25:24.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:36:38.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:35:28.000, 07/29/2025 14:38:30.000, 07/29/2025 14:39:48.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:33:53.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:37:44.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:46:00.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:45:15.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:44:25.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:47:29.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:54:48.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:53:41.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:51:26.000, 07/29/2025 14:52:44.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:51:16.000, 07/29/2025 14:55:13.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:03:00.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:01:26.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 15:00:38.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 14:57:29.000, 07/29/2025 14:58:45.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:25:22.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:26:04.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:26:51.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:28:54.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:21:23.000, 07/29/2025 16:41:49.000, 07/29/2025 16:45:04.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:42:34.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:43:22.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:44:24.000, 07/29/2025 16:45:05.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:20:29.000, 07/29/2025 16:36:20.000, 07/29/2025 16:39:16.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:37:24.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:38:15.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:38:58.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:19:19.000, 07/29/2025 16:33:33.000, 07/29/2025 16:59:34.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 17:00:18.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 17:00:56.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 17:02:00.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:46:57.000, 07/29/2025 16:48:44.000, 07/29/2025 16:50:58.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:47:26.000, 07/29/2025 16:49:18.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:47:21.000, 07/29/2025 16:49:49.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 16:47:14.000, 07/29/2025 16:50:31.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 17:09:38.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 17:07:53.000, 07/29/2025 17:10:58.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 17:07:51.000, 07/29/2025 17:12:00.000</t>
-  </si>
-  <si>
-    <t>07/29/2025 17:07:46.000</t>
   </si>
 </sst>
 </file>
@@ -569,7 +578,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:W72"/>
+  <dimension ref="A1:Y72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.5703125" customWidth="true"/>
@@ -592,9 +601,11 @@
     <col min="18" max="18" width="11.7109375" customWidth="true"/>
     <col min="19" max="19" width="9" customWidth="true"/>
     <col min="20" max="20" width="6.7109375" customWidth="true"/>
-    <col min="21" max="21" width="12" customWidth="true"/>
-    <col min="22" max="22" width="830.7109375" customWidth="true"/>
-    <col min="23" max="23" width="830.7109375" customWidth="true"/>
+    <col min="21" max="21" width="8.85546875" customWidth="true"/>
+    <col min="22" max="22" width="5.7109375" customWidth="true"/>
+    <col min="23" max="23" width="9.42578125" customWidth="true"/>
+    <col min="24" max="24" width="830.7109375" customWidth="true"/>
+    <col min="25" max="25" width="830.7109375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -662,9 +673,15 @@
         <v>23</v>
       </c>
       <c r="V1" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="W1" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="X1" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="W1" s="0" t="s">
+      <c r="Y1" s="0" t="s">
         <v>98</v>
       </c>
     </row>
@@ -730,12 +747,18 @@
         <v>1.0002</v>
       </c>
       <c r="U2" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V2" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V2" s="0">
+        <v>32</v>
+      </c>
+      <c r="W2" s="0">
+        <v>0</v>
+      </c>
+      <c r="X2" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="W2" s="0" t="s">
+      <c r="Y2" s="0" t="s">
         <v>99</v>
       </c>
     </row>
@@ -801,12 +824,18 @@
         <v>1.0002</v>
       </c>
       <c r="U3" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V3" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V3" s="0">
+        <v>32</v>
+      </c>
+      <c r="W3" s="0">
+        <v>0</v>
+      </c>
+      <c r="X3" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="W3" s="0" t="s">
+      <c r="Y3" s="0" t="s">
         <v>100</v>
       </c>
     </row>
@@ -872,12 +901,18 @@
         <v>1.0002</v>
       </c>
       <c r="U4" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V4" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V4" s="0">
+        <v>32</v>
+      </c>
+      <c r="W4" s="0">
+        <v>0</v>
+      </c>
+      <c r="X4" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="W4" s="0" t="s">
+      <c r="Y4" s="0" t="s">
         <v>101</v>
       </c>
     </row>
@@ -943,12 +978,18 @@
         <v>1.0005999999999999</v>
       </c>
       <c r="U5" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V5" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V5" s="0">
+        <v>32</v>
+      </c>
+      <c r="W5" s="0">
+        <v>50</v>
+      </c>
+      <c r="X5" s="0" t="s">
         <v>30</v>
       </c>
-      <c r="W5" s="0" t="s">
+      <c r="Y5" s="0" t="s">
         <v>102</v>
       </c>
     </row>
@@ -1014,12 +1055,18 @@
         <v>1.0005999999999999</v>
       </c>
       <c r="U6" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V6" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V6" s="0">
+        <v>32</v>
+      </c>
+      <c r="W6" s="0">
+        <v>50</v>
+      </c>
+      <c r="X6" s="0" t="s">
         <v>31</v>
       </c>
-      <c r="W6" s="0" t="s">
+      <c r="Y6" s="0" t="s">
         <v>103</v>
       </c>
     </row>
@@ -1085,12 +1132,18 @@
         <v>1.0005999999999999</v>
       </c>
       <c r="U7" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V7" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="W7" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V7" s="0">
+        <v>32</v>
+      </c>
+      <c r="W7" s="0">
+        <v>50</v>
+      </c>
+      <c r="X7" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="Y7" s="0" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1156,12 +1209,18 @@
         <v>1.0005999999999999</v>
       </c>
       <c r="U8" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V8" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V8" s="0">
+        <v>32</v>
+      </c>
+      <c r="W8" s="0">
+        <v>50</v>
+      </c>
+      <c r="X8" s="0" t="s">
         <v>33</v>
       </c>
-      <c r="W8" s="0" t="s">
+      <c r="Y8" s="0" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1227,12 +1286,18 @@
         <v>1.0024999999999999</v>
       </c>
       <c r="U9" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V9" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V9" s="0">
+        <v>32</v>
+      </c>
+      <c r="W9" s="0">
+        <v>200</v>
+      </c>
+      <c r="X9" s="0" t="s">
         <v>34</v>
       </c>
-      <c r="W9" s="0" t="s">
+      <c r="Y9" s="0" t="s">
         <v>106</v>
       </c>
     </row>
@@ -1298,12 +1363,18 @@
         <v>1.0024999999999999</v>
       </c>
       <c r="U10" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V10" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V10" s="0">
+        <v>32</v>
+      </c>
+      <c r="W10" s="0">
+        <v>200</v>
+      </c>
+      <c r="X10" s="0" t="s">
         <v>35</v>
       </c>
-      <c r="W10" s="0" t="s">
+      <c r="Y10" s="0" t="s">
         <v>107</v>
       </c>
     </row>
@@ -1369,12 +1440,18 @@
         <v>1.0024999999999999</v>
       </c>
       <c r="U11" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V11" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V11" s="0">
+        <v>32</v>
+      </c>
+      <c r="W11" s="0">
+        <v>200</v>
+      </c>
+      <c r="X11" s="0" t="s">
         <v>36</v>
       </c>
-      <c r="W11" s="0" t="s">
+      <c r="Y11" s="0" t="s">
         <v>108</v>
       </c>
     </row>
@@ -1440,12 +1517,18 @@
         <v>1.0024999999999999</v>
       </c>
       <c r="U12" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V12" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V12" s="0">
+        <v>32</v>
+      </c>
+      <c r="W12" s="0">
+        <v>200</v>
+      </c>
+      <c r="X12" s="0" t="s">
         <v>37</v>
       </c>
-      <c r="W12" s="0" t="s">
+      <c r="Y12" s="0" t="s">
         <v>109</v>
       </c>
     </row>
@@ -1511,12 +1594,18 @@
         <v>1.0063</v>
       </c>
       <c r="U13" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V13" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V13" s="0">
+        <v>32</v>
+      </c>
+      <c r="W13" s="0">
+        <v>500</v>
+      </c>
+      <c r="X13" s="0" t="s">
         <v>38</v>
       </c>
-      <c r="W13" s="0" t="s">
+      <c r="Y13" s="0" t="s">
         <v>110</v>
       </c>
     </row>
@@ -1582,12 +1671,18 @@
         <v>1.0063</v>
       </c>
       <c r="U14" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V14" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V14" s="0">
+        <v>32</v>
+      </c>
+      <c r="W14" s="0">
+        <v>500</v>
+      </c>
+      <c r="X14" s="0" t="s">
         <v>39</v>
       </c>
-      <c r="W14" s="0" t="s">
+      <c r="Y14" s="0" t="s">
         <v>111</v>
       </c>
     </row>
@@ -1653,12 +1748,18 @@
         <v>1.0063</v>
       </c>
       <c r="U15" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V15" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V15" s="0">
+        <v>32</v>
+      </c>
+      <c r="W15" s="0">
+        <v>500</v>
+      </c>
+      <c r="X15" s="0" t="s">
         <v>40</v>
       </c>
-      <c r="W15" s="0" t="s">
+      <c r="Y15" s="0" t="s">
         <v>112</v>
       </c>
     </row>
@@ -1724,12 +1825,18 @@
         <v>1.0063</v>
       </c>
       <c r="U16" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V16" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V16" s="0">
+        <v>32</v>
+      </c>
+      <c r="W16" s="0">
+        <v>500</v>
+      </c>
+      <c r="X16" s="0" t="s">
         <v>41</v>
       </c>
-      <c r="W16" s="0" t="s">
+      <c r="Y16" s="0" t="s">
         <v>113</v>
       </c>
     </row>
@@ -1795,12 +1902,18 @@
         <v>1.0126999999999999</v>
       </c>
       <c r="U17" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V17" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V17" s="0">
+        <v>32</v>
+      </c>
+      <c r="W17" s="0">
+        <v>900</v>
+      </c>
+      <c r="X17" s="0" t="s">
         <v>42</v>
       </c>
-      <c r="W17" s="0" t="s">
+      <c r="Y17" s="0" t="s">
         <v>114</v>
       </c>
     </row>
@@ -1866,12 +1979,18 @@
         <v>1.0126999999999999</v>
       </c>
       <c r="U18" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V18" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V18" s="0">
+        <v>32</v>
+      </c>
+      <c r="W18" s="0">
+        <v>900</v>
+      </c>
+      <c r="X18" s="0" t="s">
         <v>43</v>
       </c>
-      <c r="W18" s="0" t="s">
+      <c r="Y18" s="0" t="s">
         <v>115</v>
       </c>
     </row>
@@ -1937,12 +2056,18 @@
         <v>1.0126999999999999</v>
       </c>
       <c r="U19" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V19" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V19" s="0">
+        <v>32</v>
+      </c>
+      <c r="W19" s="0">
+        <v>900</v>
+      </c>
+      <c r="X19" s="0" t="s">
         <v>44</v>
       </c>
-      <c r="W19" s="0" t="s">
+      <c r="Y19" s="0" t="s">
         <v>116</v>
       </c>
     </row>
@@ -2008,12 +2133,18 @@
         <v>1.0126999999999999</v>
       </c>
       <c r="U20" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V20" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V20" s="0">
+        <v>32</v>
+      </c>
+      <c r="W20" s="0">
+        <v>900</v>
+      </c>
+      <c r="X20" s="0" t="s">
         <v>45</v>
       </c>
-      <c r="W20" s="0" t="s">
+      <c r="Y20" s="0" t="s">
         <v>117</v>
       </c>
     </row>
@@ -2079,12 +2210,18 @@
         <v>1.0237000000000001</v>
       </c>
       <c r="U21" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V21" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V21" s="0">
+        <v>32</v>
+      </c>
+      <c r="W21" s="0">
+        <v>1500</v>
+      </c>
+      <c r="X21" s="0" t="s">
         <v>46</v>
       </c>
-      <c r="W21" s="0" t="s">
+      <c r="Y21" s="0" t="s">
         <v>118</v>
       </c>
     </row>
@@ -2150,12 +2287,18 @@
         <v>1.0237000000000001</v>
       </c>
       <c r="U22" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V22" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V22" s="0">
+        <v>32</v>
+      </c>
+      <c r="W22" s="0">
+        <v>1500</v>
+      </c>
+      <c r="X22" s="0" t="s">
         <v>47</v>
       </c>
-      <c r="W22" s="0" t="s">
+      <c r="Y22" s="0" t="s">
         <v>119</v>
       </c>
     </row>
@@ -2221,12 +2364,18 @@
         <v>1.0237000000000001</v>
       </c>
       <c r="U23" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V23" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V23" s="0">
+        <v>32</v>
+      </c>
+      <c r="W23" s="0">
+        <v>1500</v>
+      </c>
+      <c r="X23" s="0" t="s">
         <v>48</v>
       </c>
-      <c r="W23" s="0" t="s">
+      <c r="Y23" s="0" t="s">
         <v>120</v>
       </c>
     </row>
@@ -2292,12 +2441,18 @@
         <v>1.0237000000000001</v>
       </c>
       <c r="U24" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V24" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="V24" s="0">
+        <v>32</v>
+      </c>
+      <c r="W24" s="0">
+        <v>1500</v>
+      </c>
+      <c r="X24" s="0" t="s">
         <v>49</v>
       </c>
-      <c r="W24" s="0" t="s">
+      <c r="Y24" s="0" t="s">
         <v>121</v>
       </c>
     </row>
@@ -2363,12 +2518,18 @@
         <v>1.0003</v>
       </c>
       <c r="U25" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V25" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V25" s="0">
+        <v>32</v>
+      </c>
+      <c r="W25" s="0">
+        <v>0</v>
+      </c>
+      <c r="X25" s="0" t="s">
         <v>50</v>
       </c>
-      <c r="W25" s="0" t="s">
+      <c r="Y25" s="0" t="s">
         <v>122</v>
       </c>
     </row>
@@ -2434,12 +2595,18 @@
         <v>1.0003</v>
       </c>
       <c r="U26" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V26" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V26" s="0">
+        <v>32</v>
+      </c>
+      <c r="W26" s="0">
+        <v>0</v>
+      </c>
+      <c r="X26" s="0" t="s">
         <v>51</v>
       </c>
-      <c r="W26" s="0" t="s">
+      <c r="Y26" s="0" t="s">
         <v>123</v>
       </c>
     </row>
@@ -2505,12 +2672,18 @@
         <v>1.0003</v>
       </c>
       <c r="U27" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V27" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V27" s="0">
+        <v>32</v>
+      </c>
+      <c r="W27" s="0">
+        <v>0</v>
+      </c>
+      <c r="X27" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="W27" s="0" t="s">
+      <c r="Y27" s="0" t="s">
         <v>124</v>
       </c>
     </row>
@@ -2576,12 +2749,18 @@
         <v>1.0003</v>
       </c>
       <c r="U28" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V28" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V28" s="0">
+        <v>32</v>
+      </c>
+      <c r="W28" s="0">
+        <v>0</v>
+      </c>
+      <c r="X28" s="0" t="s">
         <v>53</v>
       </c>
-      <c r="W28" s="0" t="s">
+      <c r="Y28" s="0" t="s">
         <v>125</v>
       </c>
     </row>
@@ -2647,12 +2826,18 @@
         <v>1.0011000000000001</v>
       </c>
       <c r="U29" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V29" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V29" s="0">
+        <v>32</v>
+      </c>
+      <c r="W29" s="0">
+        <v>50</v>
+      </c>
+      <c r="X29" s="0" t="s">
         <v>54</v>
       </c>
-      <c r="W29" s="0" t="s">
+      <c r="Y29" s="0" t="s">
         <v>126</v>
       </c>
     </row>
@@ -2718,12 +2903,18 @@
         <v>1.0011000000000001</v>
       </c>
       <c r="U30" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V30" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V30" s="0">
+        <v>32</v>
+      </c>
+      <c r="W30" s="0">
+        <v>50</v>
+      </c>
+      <c r="X30" s="0" t="s">
         <v>55</v>
       </c>
-      <c r="W30" s="0" t="s">
+      <c r="Y30" s="0" t="s">
         <v>127</v>
       </c>
     </row>
@@ -2789,12 +2980,18 @@
         <v>1.0011000000000001</v>
       </c>
       <c r="U31" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V31" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V31" s="0">
+        <v>32</v>
+      </c>
+      <c r="W31" s="0">
+        <v>50</v>
+      </c>
+      <c r="X31" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="W31" s="0" t="s">
+      <c r="Y31" s="0" t="s">
         <v>128</v>
       </c>
     </row>
@@ -2860,12 +3057,18 @@
         <v>1.0011000000000001</v>
       </c>
       <c r="U32" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V32" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V32" s="0">
+        <v>32</v>
+      </c>
+      <c r="W32" s="0">
+        <v>50</v>
+      </c>
+      <c r="X32" s="0" t="s">
         <v>57</v>
       </c>
-      <c r="W32" s="0" t="s">
+      <c r="Y32" s="0" t="s">
         <v>129</v>
       </c>
     </row>
@@ -2931,12 +3134,18 @@
         <v>1.0043</v>
       </c>
       <c r="U33" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V33" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V33" s="0">
+        <v>32</v>
+      </c>
+      <c r="W33" s="0">
+        <v>200</v>
+      </c>
+      <c r="X33" s="0" t="s">
         <v>58</v>
       </c>
-      <c r="W33" s="0" t="s">
+      <c r="Y33" s="0" t="s">
         <v>130</v>
       </c>
     </row>
@@ -3002,12 +3211,18 @@
         <v>1.0043</v>
       </c>
       <c r="U34" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V34" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V34" s="0">
+        <v>32</v>
+      </c>
+      <c r="W34" s="0">
+        <v>200</v>
+      </c>
+      <c r="X34" s="0" t="s">
         <v>59</v>
       </c>
-      <c r="W34" s="0" t="s">
+      <c r="Y34" s="0" t="s">
         <v>131</v>
       </c>
     </row>
@@ -3073,12 +3288,18 @@
         <v>1.0043</v>
       </c>
       <c r="U35" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V35" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V35" s="0">
+        <v>32</v>
+      </c>
+      <c r="W35" s="0">
+        <v>200</v>
+      </c>
+      <c r="X35" s="0" t="s">
         <v>60</v>
       </c>
-      <c r="W35" s="0" t="s">
+      <c r="Y35" s="0" t="s">
         <v>132</v>
       </c>
     </row>
@@ -3144,12 +3365,18 @@
         <v>1.0043</v>
       </c>
       <c r="U36" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V36" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V36" s="0">
+        <v>32</v>
+      </c>
+      <c r="W36" s="0">
+        <v>200</v>
+      </c>
+      <c r="X36" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="W36" s="0" t="s">
+      <c r="Y36" s="0" t="s">
         <v>133</v>
       </c>
     </row>
@@ -3215,12 +3442,18 @@
         <v>1.0105999999999999</v>
       </c>
       <c r="U37" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V37" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V37" s="0">
+        <v>32</v>
+      </c>
+      <c r="W37" s="0">
+        <v>500</v>
+      </c>
+      <c r="X37" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="W37" s="0" t="s">
+      <c r="Y37" s="0" t="s">
         <v>134</v>
       </c>
     </row>
@@ -3286,12 +3519,18 @@
         <v>1.0105999999999999</v>
       </c>
       <c r="U38" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V38" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V38" s="0">
+        <v>32</v>
+      </c>
+      <c r="W38" s="0">
+        <v>500</v>
+      </c>
+      <c r="X38" s="0" t="s">
         <v>63</v>
       </c>
-      <c r="W38" s="0" t="s">
+      <c r="Y38" s="0" t="s">
         <v>135</v>
       </c>
     </row>
@@ -3357,12 +3596,18 @@
         <v>1.0105999999999999</v>
       </c>
       <c r="U39" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V39" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V39" s="0">
+        <v>32</v>
+      </c>
+      <c r="W39" s="0">
+        <v>500</v>
+      </c>
+      <c r="X39" s="0" t="s">
         <v>64</v>
       </c>
-      <c r="W39" s="0" t="s">
+      <c r="Y39" s="0" t="s">
         <v>136</v>
       </c>
     </row>
@@ -3428,12 +3673,18 @@
         <v>1.0105999999999999</v>
       </c>
       <c r="U40" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V40" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V40" s="0">
+        <v>32</v>
+      </c>
+      <c r="W40" s="0">
+        <v>500</v>
+      </c>
+      <c r="X40" s="0" t="s">
         <v>65</v>
       </c>
-      <c r="W40" s="0" t="s">
+      <c r="Y40" s="0" t="s">
         <v>137</v>
       </c>
     </row>
@@ -3499,12 +3750,18 @@
         <v>1.0204</v>
       </c>
       <c r="U41" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V41" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V41" s="0">
+        <v>32</v>
+      </c>
+      <c r="W41" s="0">
+        <v>900</v>
+      </c>
+      <c r="X41" s="0" t="s">
         <v>66</v>
       </c>
-      <c r="W41" s="0" t="s">
+      <c r="Y41" s="0" t="s">
         <v>138</v>
       </c>
     </row>
@@ -3570,12 +3827,18 @@
         <v>1.0204</v>
       </c>
       <c r="U42" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V42" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V42" s="0">
+        <v>32</v>
+      </c>
+      <c r="W42" s="0">
+        <v>900</v>
+      </c>
+      <c r="X42" s="0" t="s">
         <v>67</v>
       </c>
-      <c r="W42" s="0" t="s">
+      <c r="Y42" s="0" t="s">
         <v>139</v>
       </c>
     </row>
@@ -3641,12 +3904,18 @@
         <v>1.0204</v>
       </c>
       <c r="U43" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V43" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V43" s="0">
+        <v>32</v>
+      </c>
+      <c r="W43" s="0">
+        <v>900</v>
+      </c>
+      <c r="X43" s="0" t="s">
         <v>68</v>
       </c>
-      <c r="W43" s="0" t="s">
+      <c r="Y43" s="0" t="s">
         <v>140</v>
       </c>
     </row>
@@ -3712,12 +3981,18 @@
         <v>1.0204</v>
       </c>
       <c r="U44" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V44" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V44" s="0">
+        <v>32</v>
+      </c>
+      <c r="W44" s="0">
+        <v>900</v>
+      </c>
+      <c r="X44" s="0" t="s">
         <v>69</v>
       </c>
-      <c r="W44" s="0" t="s">
+      <c r="Y44" s="0" t="s">
         <v>141</v>
       </c>
     </row>
@@ -3783,12 +4058,18 @@
         <v>1.0364</v>
       </c>
       <c r="U45" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V45" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V45" s="0">
+        <v>32</v>
+      </c>
+      <c r="W45" s="0">
+        <v>1500</v>
+      </c>
+      <c r="X45" s="0" t="s">
         <v>70</v>
       </c>
-      <c r="W45" s="0" t="s">
+      <c r="Y45" s="0" t="s">
         <v>142</v>
       </c>
     </row>
@@ -3854,12 +4135,18 @@
         <v>1.0364</v>
       </c>
       <c r="U46" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V46" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V46" s="0">
+        <v>32</v>
+      </c>
+      <c r="W46" s="0">
+        <v>1500</v>
+      </c>
+      <c r="X46" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="W46" s="0" t="s">
+      <c r="Y46" s="0" t="s">
         <v>143</v>
       </c>
     </row>
@@ -3925,12 +4212,18 @@
         <v>1.0364</v>
       </c>
       <c r="U47" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V47" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V47" s="0">
+        <v>32</v>
+      </c>
+      <c r="W47" s="0">
+        <v>1500</v>
+      </c>
+      <c r="X47" s="0" t="s">
         <v>72</v>
       </c>
-      <c r="W47" s="0" t="s">
+      <c r="Y47" s="0" t="s">
         <v>144</v>
       </c>
     </row>
@@ -3996,12 +4289,18 @@
         <v>1.0364</v>
       </c>
       <c r="U48" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V48" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="V48" s="0">
+        <v>32</v>
+      </c>
+      <c r="W48" s="0">
+        <v>1500</v>
+      </c>
+      <c r="X48" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="W48" s="0" t="s">
+      <c r="Y48" s="0" t="s">
         <v>145</v>
       </c>
     </row>
@@ -4067,12 +4366,18 @@
         <v>0.99490000000000001</v>
       </c>
       <c r="U49" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V49" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V49" s="0">
+        <v>32</v>
+      </c>
+      <c r="W49" s="0">
+        <v>0</v>
+      </c>
+      <c r="X49" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="W49" s="0" t="s">
+      <c r="Y49" s="0" t="s">
         <v>146</v>
       </c>
     </row>
@@ -4138,12 +4443,18 @@
         <v>0.99490000000000001</v>
       </c>
       <c r="U50" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V50" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V50" s="0">
+        <v>32</v>
+      </c>
+      <c r="W50" s="0">
+        <v>0</v>
+      </c>
+      <c r="X50" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="W50" s="0" t="s">
+      <c r="Y50" s="0" t="s">
         <v>147</v>
       </c>
     </row>
@@ -4209,12 +4520,18 @@
         <v>0.99490000000000001</v>
       </c>
       <c r="U51" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V51" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V51" s="0">
+        <v>32</v>
+      </c>
+      <c r="W51" s="0">
+        <v>0</v>
+      </c>
+      <c r="X51" s="0" t="s">
         <v>76</v>
       </c>
-      <c r="W51" s="0" t="s">
+      <c r="Y51" s="0" t="s">
         <v>148</v>
       </c>
     </row>
@@ -4280,12 +4597,18 @@
         <v>0.99490000000000001</v>
       </c>
       <c r="U52" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V52" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V52" s="0">
+        <v>32</v>
+      </c>
+      <c r="W52" s="0">
+        <v>0</v>
+      </c>
+      <c r="X52" s="0" t="s">
         <v>77</v>
       </c>
-      <c r="W52" s="0" t="s">
+      <c r="Y52" s="0" t="s">
         <v>149</v>
       </c>
     </row>
@@ -4351,12 +4674,18 @@
         <v>0.97940000000000005</v>
       </c>
       <c r="U53" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V53" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V53" s="0">
+        <v>32</v>
+      </c>
+      <c r="W53" s="0">
+        <v>50</v>
+      </c>
+      <c r="X53" s="0" t="s">
         <v>78</v>
       </c>
-      <c r="W53" s="0" t="s">
+      <c r="Y53" s="0" t="s">
         <v>150</v>
       </c>
     </row>
@@ -4422,12 +4751,18 @@
         <v>0.97940000000000005</v>
       </c>
       <c r="U54" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V54" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V54" s="0">
+        <v>32</v>
+      </c>
+      <c r="W54" s="0">
+        <v>50</v>
+      </c>
+      <c r="X54" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="W54" s="0" t="s">
+      <c r="Y54" s="0" t="s">
         <v>151</v>
       </c>
     </row>
@@ -4493,12 +4828,18 @@
         <v>0.97940000000000005</v>
       </c>
       <c r="U55" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V55" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V55" s="0">
+        <v>32</v>
+      </c>
+      <c r="W55" s="0">
+        <v>50</v>
+      </c>
+      <c r="X55" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="W55" s="0" t="s">
+      <c r="Y55" s="0" t="s">
         <v>152</v>
       </c>
     </row>
@@ -4564,12 +4905,18 @@
         <v>0.97940000000000005</v>
       </c>
       <c r="U56" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V56" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V56" s="0">
+        <v>32</v>
+      </c>
+      <c r="W56" s="0">
+        <v>50</v>
+      </c>
+      <c r="X56" s="0" t="s">
         <v>81</v>
       </c>
-      <c r="W56" s="0" t="s">
+      <c r="Y56" s="0" t="s">
         <v>153</v>
       </c>
     </row>
@@ -4635,12 +4982,18 @@
         <v>0.92059999999999997</v>
       </c>
       <c r="U57" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V57" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V57" s="0">
+        <v>32</v>
+      </c>
+      <c r="W57" s="0">
+        <v>200</v>
+      </c>
+      <c r="X57" s="0" t="s">
         <v>82</v>
       </c>
-      <c r="W57" s="0" t="s">
+      <c r="Y57" s="0" t="s">
         <v>154</v>
       </c>
     </row>
@@ -4706,12 +5059,18 @@
         <v>0.92059999999999997</v>
       </c>
       <c r="U58" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V58" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V58" s="0">
+        <v>32</v>
+      </c>
+      <c r="W58" s="0">
+        <v>200</v>
+      </c>
+      <c r="X58" s="0" t="s">
         <v>83</v>
       </c>
-      <c r="W58" s="0" t="s">
+      <c r="Y58" s="0" t="s">
         <v>155</v>
       </c>
     </row>
@@ -4777,12 +5136,18 @@
         <v>0.92059999999999997</v>
       </c>
       <c r="U59" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V59" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V59" s="0">
+        <v>32</v>
+      </c>
+      <c r="W59" s="0">
+        <v>200</v>
+      </c>
+      <c r="X59" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="W59" s="0" t="s">
+      <c r="Y59" s="0" t="s">
         <v>156</v>
       </c>
     </row>
@@ -4848,12 +5213,18 @@
         <v>0.92059999999999997</v>
       </c>
       <c r="U60" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V60" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V60" s="0">
+        <v>32</v>
+      </c>
+      <c r="W60" s="0">
+        <v>200</v>
+      </c>
+      <c r="X60" s="0" t="s">
         <v>85</v>
       </c>
-      <c r="W60" s="0" t="s">
+      <c r="Y60" s="0" t="s">
         <v>157</v>
       </c>
     </row>
@@ -4919,12 +5290,18 @@
         <v>0.80210000000000004</v>
       </c>
       <c r="U61" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V61" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V61" s="0">
+        <v>32</v>
+      </c>
+      <c r="W61" s="0">
+        <v>500</v>
+      </c>
+      <c r="X61" s="0" t="s">
         <v>86</v>
       </c>
-      <c r="W61" s="0" t="s">
+      <c r="Y61" s="0" t="s">
         <v>158</v>
       </c>
     </row>
@@ -4990,12 +5367,18 @@
         <v>0.80210000000000004</v>
       </c>
       <c r="U62" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V62" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V62" s="0">
+        <v>32</v>
+      </c>
+      <c r="W62" s="0">
+        <v>500</v>
+      </c>
+      <c r="X62" s="0" t="s">
         <v>87</v>
       </c>
-      <c r="W62" s="0" t="s">
+      <c r="Y62" s="0" t="s">
         <v>159</v>
       </c>
     </row>
@@ -5061,12 +5444,18 @@
         <v>0.80210000000000004</v>
       </c>
       <c r="U63" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V63" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V63" s="0">
+        <v>32</v>
+      </c>
+      <c r="W63" s="0">
+        <v>500</v>
+      </c>
+      <c r="X63" s="0" t="s">
         <v>88</v>
       </c>
-      <c r="W63" s="0" t="s">
+      <c r="Y63" s="0" t="s">
         <v>160</v>
       </c>
     </row>
@@ -5132,12 +5521,18 @@
         <v>0.80210000000000004</v>
       </c>
       <c r="U64" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V64" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V64" s="0">
+        <v>32</v>
+      </c>
+      <c r="W64" s="0">
+        <v>500</v>
+      </c>
+      <c r="X64" s="0" t="s">
         <v>89</v>
       </c>
-      <c r="W64" s="0" t="s">
+      <c r="Y64" s="0" t="s">
         <v>161</v>
       </c>
     </row>
@@ -5203,12 +5598,18 @@
         <v>0.57979999999999998</v>
       </c>
       <c r="U65" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V65" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V65" s="0">
+        <v>32</v>
+      </c>
+      <c r="W65" s="0">
+        <v>900</v>
+      </c>
+      <c r="X65" s="0" t="s">
         <v>90</v>
       </c>
-      <c r="W65" s="0" t="s">
+      <c r="Y65" s="0" t="s">
         <v>162</v>
       </c>
     </row>
@@ -5274,12 +5675,18 @@
         <v>0.57979999999999998</v>
       </c>
       <c r="U66" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V66" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V66" s="0">
+        <v>32</v>
+      </c>
+      <c r="W66" s="0">
+        <v>900</v>
+      </c>
+      <c r="X66" s="0" t="s">
         <v>91</v>
       </c>
-      <c r="W66" s="0" t="s">
+      <c r="Y66" s="0" t="s">
         <v>163</v>
       </c>
     </row>
@@ -5345,12 +5752,18 @@
         <v>0.57979999999999998</v>
       </c>
       <c r="U67" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V67" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V67" s="0">
+        <v>32</v>
+      </c>
+      <c r="W67" s="0">
+        <v>900</v>
+      </c>
+      <c r="X67" s="0" t="s">
         <v>92</v>
       </c>
-      <c r="W67" s="0" t="s">
+      <c r="Y67" s="0" t="s">
         <v>164</v>
       </c>
     </row>
@@ -5416,12 +5829,18 @@
         <v>0.57979999999999998</v>
       </c>
       <c r="U68" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="V68" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V68" s="0">
+        <v>32</v>
+      </c>
+      <c r="W68" s="0">
+        <v>900</v>
+      </c>
+      <c r="X68" s="0" t="s">
         <v>93</v>
       </c>
-      <c r="W68" s="0" t="s">
+      <c r="Y68" s="0" t="s">
         <v>165</v>
       </c>
     </row>
@@ -5487,12 +5906,18 @@
         <v>0.25430000000000003</v>
       </c>
       <c r="U69" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V69" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V69" s="0">
+        <v>32</v>
+      </c>
+      <c r="W69" s="0">
+        <v>1500</v>
+      </c>
+      <c r="X69" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="W69" s="0" t="s">
+      <c r="Y69" s="0" t="s">
         <v>166</v>
       </c>
     </row>
@@ -5558,12 +5983,18 @@
         <v>0.25430000000000003</v>
       </c>
       <c r="U70" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V70" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V70" s="0">
+        <v>32</v>
+      </c>
+      <c r="W70" s="0">
+        <v>1500</v>
+      </c>
+      <c r="X70" s="0" t="s">
         <v>95</v>
       </c>
-      <c r="W70" s="0" t="s">
+      <c r="Y70" s="0" t="s">
         <v>167</v>
       </c>
     </row>
@@ -5629,12 +6060,18 @@
         <v>0.25430000000000003</v>
       </c>
       <c r="U71" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V71" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V71" s="0">
+        <v>32</v>
+      </c>
+      <c r="W71" s="0">
+        <v>1500</v>
+      </c>
+      <c r="X71" s="0" t="s">
         <v>96</v>
       </c>
-      <c r="W71" s="0" t="s">
+      <c r="Y71" s="0" t="s">
         <v>168</v>
       </c>
     </row>
@@ -5700,12 +6137,18 @@
         <v>0.25430000000000003</v>
       </c>
       <c r="U72" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="V72" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="V72" s="0">
+        <v>32</v>
+      </c>
+      <c r="W72" s="0">
+        <v>1500</v>
+      </c>
+      <c r="X72" s="0" t="s">
         <v>97</v>
       </c>
-      <c r="W72" s="0" t="s">
+      <c r="Y72" s="0" t="s">
         <v>169</v>
       </c>
     </row>
@@ -5811,7 +6254,7 @@
         <v>22</v>
       </c>
       <c r="W1" t="s">
-        <v>23</v>
+        <v>170</v>
       </c>
     </row>
     <row r="2">
@@ -5878,7 +6321,7 @@
         <v>1.0002</v>
       </c>
       <c r="W2" t="s">
-        <v>24</v>
+        <v>171</v>
       </c>
     </row>
     <row r="3">
@@ -5945,7 +6388,7 @@
         <v>1.0005999999999999</v>
       </c>
       <c r="W3" t="s">
-        <v>25</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4">
@@ -6012,7 +6455,7 @@
         <v>1.0024999999999999</v>
       </c>
       <c r="W4" t="s">
-        <v>25</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5">
@@ -6079,7 +6522,7 @@
         <v>1.0063</v>
       </c>
       <c r="W5" t="s">
-        <v>25</v>
+        <v>172</v>
       </c>
     </row>
     <row r="6">
@@ -6146,7 +6589,7 @@
         <v>1.0126999999999999</v>
       </c>
       <c r="W6" t="s">
-        <v>25</v>
+        <v>172</v>
       </c>
     </row>
     <row r="7">
@@ -6213,7 +6656,7 @@
         <v>1.0237000000000001</v>
       </c>
       <c r="W7" t="s">
-        <v>25</v>
+        <v>172</v>
       </c>
     </row>
     <row r="8">
@@ -6280,7 +6723,7 @@
         <v>1.0003</v>
       </c>
       <c r="W8" t="s">
-        <v>24</v>
+        <v>171</v>
       </c>
     </row>
     <row r="9">
@@ -6347,7 +6790,7 @@
         <v>1.0011000000000001</v>
       </c>
       <c r="W9" t="s">
-        <v>24</v>
+        <v>171</v>
       </c>
     </row>
     <row r="10">
@@ -6414,7 +6857,7 @@
         <v>1.0043</v>
       </c>
       <c r="W10" t="s">
-        <v>25</v>
+        <v>172</v>
       </c>
     </row>
     <row r="11">
@@ -6481,7 +6924,7 @@
         <v>1.0105999999999999</v>
       </c>
       <c r="W11" t="s">
-        <v>25</v>
+        <v>172</v>
       </c>
     </row>
     <row r="12">
@@ -6548,7 +6991,7 @@
         <v>1.0204</v>
       </c>
       <c r="W12" t="s">
-        <v>25</v>
+        <v>172</v>
       </c>
     </row>
     <row r="13">
@@ -6615,7 +7058,7 @@
         <v>1.0364</v>
       </c>
       <c r="W13" t="s">
-        <v>25</v>
+        <v>172</v>
       </c>
     </row>
     <row r="14">
@@ -6682,7 +7125,7 @@
         <v>0.99490000000000001</v>
       </c>
       <c r="W14" t="s">
-        <v>24</v>
+        <v>171</v>
       </c>
     </row>
     <row r="15">
@@ -6749,7 +7192,7 @@
         <v>0.97940000000000005</v>
       </c>
       <c r="W15" t="s">
-        <v>24</v>
+        <v>171</v>
       </c>
     </row>
     <row r="16">
@@ -6816,7 +7259,7 @@
         <v>0.92059999999999997</v>
       </c>
       <c r="W16" t="s">
-        <v>24</v>
+        <v>171</v>
       </c>
     </row>
     <row r="17">
@@ -6883,7 +7326,7 @@
         <v>0.80210000000000004</v>
       </c>
       <c r="W17" t="s">
-        <v>24</v>
+        <v>171</v>
       </c>
     </row>
     <row r="18">
@@ -6950,7 +7393,7 @@
         <v>0.57979999999999998</v>
       </c>
       <c r="W18" t="s">
-        <v>24</v>
+        <v>171</v>
       </c>
     </row>
     <row r="19">
@@ -7017,7 +7460,7 @@
         <v>0.25430000000000003</v>
       </c>
       <c r="W19" t="s">
-        <v>25</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>

</xml_diff>